<commit_message>
Datos al 23-10-2026, montos en texto en hojas de Brecha y exportables nuevos
- Excel actualizado al 23-10-2026 y panel regenerado.
- Brechas: to_float entiende montos como texto ("CLP 343.081"); Sin Stock y
  Oport. por Facturar salían en 0.
- Matriz de Prospección: el Excel exportado trae además las hojas
  Consolidado y Carta Gantt del Plan de Visitas.
- Visitas: botón Exportar en Cobertura por Ejecutivo y Visitas Mensuales.
- Presentación 20261023, Clientes_puntuales y Top 10 Metropolitana sin VACIO.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Clientes_puntuales.xlsx
+++ b/Clientes_puntuales.xlsx
@@ -1,160 +1,82 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cmuñoz\Desktop\Panel-TECSERVICE\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55083539-CF0D-4925-A85C-1CFF18DED3CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Clientes Puntuales" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes Puntuales" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
-  <si>
-    <t>#</t>
-  </si>
-  <si>
-    <t>Cliente</t>
-  </si>
-  <si>
-    <t>Pot. ST anual MM$</t>
-  </si>
-  <si>
-    <t>Región</t>
-  </si>
-  <si>
-    <t>Base Instalada Total</t>
-  </si>
-  <si>
-    <t>Base Instalada Total (Potencial TS)</t>
-  </si>
-  <si>
-    <t>Facturación 2026</t>
-  </si>
-  <si>
-    <t>Facturación 2025</t>
-  </si>
-  <si>
-    <t>Estado</t>
-  </si>
-  <si>
-    <t>Clínica Sanatorio Alemán</t>
-  </si>
-  <si>
-    <t>Hospital Guillermo Grant Benavente</t>
-  </si>
-  <si>
-    <t>Hospital Penco Lirquén</t>
-  </si>
-  <si>
-    <t>Hospital Pitrufquén</t>
-  </si>
-  <si>
-    <t>Hospital Víctor Ríos Ruiz</t>
-  </si>
-  <si>
-    <t>Clínica Bío Bío</t>
-  </si>
-  <si>
-    <t>Hospital de Talcahuano (Las Higueras)</t>
-  </si>
-  <si>
-    <t>Bío Bío</t>
-  </si>
-  <si>
-    <t>Araucanía</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="166" formatCode="#,##0;\-#,##0;&quot;–&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0;\-#,##0;&quot;–&quot;"/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
+      <name val="Calibri"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
-      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <sz val="9"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <sz val="9"/>
     </font>
     <font>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="7">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -299,68 +221,136 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="19">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Millares [0]" xfId="1" builtinId="6"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -685,265 +675,312 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.85546875" customWidth="1"/>
+    <col width="3.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="31.85546875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="16.42578125" customWidth="1" min="3" max="3"/>
+    <col hidden="1" width="12.42578125" customWidth="1" min="4" max="4"/>
+    <col hidden="1" width="18.5703125" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12.85546875" customWidth="1" min="7" max="7"/>
+    <col width="14.28515625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="36.85546875" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="6" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" ht="30" customFormat="1" customHeight="1" s="6">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Región</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Base Instalada Total</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Base Instalada Total (Potencial TS)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Facturación 2026</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Facturación 2025</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Pot. ST anual MM$</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Hospital Guillermo Grant Benavente</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Bío Bío</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E2" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F2" s="16" t="n">
+        <v>9767515</v>
+      </c>
+      <c r="G2" s="16" t="n">
+        <v>14213737</v>
+      </c>
+      <c r="H2" s="16" t="n">
+        <v>26722485</v>
+      </c>
+      <c r="I2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Hospital Pitrufquén</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Araucanía</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>31189544</v>
+      </c>
+      <c r="G3" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="H3" s="16" t="n">
+        <v>10216195</v>
+      </c>
+      <c r="I3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Hospital Penco Lirquén</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Bío Bío</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F4" s="16" t="n">
+        <v>11835530</v>
+      </c>
+      <c r="G4" s="16" t="n">
+        <v>10809369</v>
+      </c>
+      <c r="H4" s="16" t="n">
+        <v>16345912</v>
+      </c>
+      <c r="I4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Hospital Víctor Ríos Ruiz</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Bío Bío</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>106</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>45</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>8499051</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>40564842</v>
+      </c>
+      <c r="I5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Clínica Bío Bío</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Bío Bío</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>6450708</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>8579403</v>
+      </c>
+      <c r="I6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Clínica Sanatorio Alemán</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Bío Bío</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>6156061</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>26642795</v>
+      </c>
+      <c r="I7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>8</v>
-      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Hospital de Talcahuano (Las Higueras)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Bío Bío</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <v>4699149</v>
+      </c>
+      <c r="I8" s="8" t="n"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="12">
-        <v>20</v>
-      </c>
-      <c r="E2" s="12">
-        <v>15</v>
-      </c>
-      <c r="F2" s="15">
-        <v>25485358</v>
-      </c>
-      <c r="G2" s="15">
-        <v>14213737</v>
-      </c>
-      <c r="H2" s="15">
-        <v>24925315</v>
-      </c>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="12">
-        <v>13</v>
-      </c>
-      <c r="E3" s="12">
-        <v>5</v>
-      </c>
-      <c r="F3" s="15">
-        <v>24282977</v>
-      </c>
-      <c r="G3" s="15">
-        <v>402732</v>
-      </c>
-      <c r="H3" s="15">
-        <v>10216195</v>
-      </c>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="12">
-        <v>28</v>
-      </c>
-      <c r="E4" s="12">
-        <v>8</v>
-      </c>
-      <c r="F4" s="15">
-        <v>10253258</v>
-      </c>
-      <c r="G4" s="15">
-        <v>10809369</v>
-      </c>
-      <c r="H4" s="15">
-        <v>16345912</v>
-      </c>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="12">
-        <v>106</v>
-      </c>
-      <c r="E5" s="12">
-        <v>45</v>
-      </c>
-      <c r="F5" s="15">
-        <v>8551286</v>
-      </c>
-      <c r="G5" s="15">
-        <v>6711156</v>
-      </c>
-      <c r="H5" s="15">
-        <v>37869087</v>
-      </c>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="12">
-        <v>7</v>
-      </c>
-      <c r="E6" s="12">
-        <v>7</v>
-      </c>
-      <c r="F6" s="15">
-        <v>5959997</v>
-      </c>
-      <c r="G6" s="15">
-        <v>0</v>
-      </c>
-      <c r="H6" s="15">
-        <v>8579403</v>
-      </c>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="12">
-        <v>16</v>
-      </c>
-      <c r="E7" s="12">
-        <v>15</v>
-      </c>
-      <c r="F7" s="15">
-        <v>1338767</v>
-      </c>
-      <c r="G7" s="15">
-        <v>4473351</v>
-      </c>
-      <c r="H7" s="15">
-        <v>26642795</v>
-      </c>
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
-        <v>7</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="13">
-        <v>12</v>
-      </c>
-      <c r="E8" s="13">
-        <v>3</v>
-      </c>
-      <c r="F8" s="14">
-        <v>0</v>
-      </c>
-      <c r="G8" s="14">
-        <v>0</v>
-      </c>
-      <c r="H8" s="14">
-        <v>4699149</v>
-      </c>
-      <c r="I8" s="8"/>
-    </row>
-    <row r="9" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" customFormat="1" s="9">
       <c r="D9" s="10">
         <f>+SUM(D2:D8)</f>
-        <v>202</v>
+        <v/>
       </c>
       <c r="E9" s="10">
         <f>+SUM(E2:E8)</f>
-        <v>98</v>
-      </c>
-      <c r="F9" s="11">
+        <v/>
+      </c>
+      <c r="F9" s="18">
         <f>+SUM(F2:F8)</f>
-        <v>75871643</v>
-      </c>
-      <c r="G9" s="11">
+        <v/>
+      </c>
+      <c r="G9" s="18">
         <f>+SUM(G2:G8)</f>
-        <v>36610345</v>
-      </c>
-      <c r="H9" s="11">
+        <v/>
+      </c>
+      <c r="H9" s="18">
         <f>+SUM(H2:H8)</f>
-        <v>129277856</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:B1 A2 A3 A4 A5 A6 A7 A8 H1" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>